<commit_message>
Updated .gitignore and added vis
</commit_message>
<xml_diff>
--- a/outputs/prolongation_report_2023.xlsx
+++ b/outputs/prolongation_report_2023.xlsx
@@ -11,7 +11,8 @@
     <sheet name="1_manager_kpi_yearly" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2_department_kpi" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="2_department_yearly" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="4_visuals" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="3_diagnostics" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="4_visuals" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6113,6 +6114,237 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>total_projects</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>excluded_stop_end</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>used_prev_month_fallback</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>excluded_share</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Васильев Артем Александрович</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>139</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.1366906474820144</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Иванова Мария Сергеевна</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>48</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.1041666666666667</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Кузнецов Михаил Иванович</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>23</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.08695652173913043</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Михайлов Андрей Сергеевич</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>31</v>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.09677419354838709</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Петрова Анна Дмитриевна</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Попова Екатерина Николаевна</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>76</v>
+      </c>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.06578947368421052</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Смирнова Ольга Владимировна</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>69</v>
+      </c>
+      <c r="C8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.1449275362318841</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Соколова Анастасия Викторовна</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>86</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.04651162790697674</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Федорова Марина Васильевна</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>без А/М</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>